<commit_message>
Force GitHub Pages rebuild
</commit_message>
<xml_diff>
--- a/Spot_Hire_Update_20260611.xlsx
+++ b/Spot_Hire_Update_20260611.xlsx
@@ -2,29 +2,46 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://my.shell.com/personal/chris_coyle_shell_com/Documents/VS Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="11_C9588FE751541D8D1C6E4DD53657CAD1CCF10B9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58FFBD33-0749-43B0-A40B-262707EBE866}"/>
+  <xr:revisionPtr revIDLastSave="618" documentId="11_C9588FE751541D8D1C6E4DD53657CAD1CCF10B9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CEB083B-588E-4873-9E7E-A46681CBC432}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spot Hire Update" sheetId="1" r:id="rId1"/>
     <sheet name="Reference" sheetId="2" r:id="rId2"/>
+    <sheet name="Asset Pivot" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Spot Hire Update'!$A$1:$I$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Spot Hire Update'!$A$1:$I$71</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId4"/>
+  </pivotCaches>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="97">
   <si>
     <t>Asset</t>
   </si>
@@ -245,9 +262,6 @@
     <t>Princess P8 Sidetrack</t>
   </si>
   <si>
-    <t xml:space="preserve">P13 Top Hole </t>
-  </si>
-  <si>
     <t>Kaikias KI-2 Drill New Well</t>
   </si>
   <si>
@@ -276,6 +290,48 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>UWX1 Deepen Hole</t>
+  </si>
+  <si>
+    <t>Princess P8 Completion</t>
+  </si>
+  <si>
+    <t>Ursa North P013 Deepening</t>
+  </si>
+  <si>
+    <t>Ursa</t>
+  </si>
+  <si>
+    <t>Sparta SP106 Deepen Hole</t>
+  </si>
+  <si>
+    <t>Ursa North P013 Top Hole</t>
+  </si>
+  <si>
+    <t>Highest Vessel Count</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Highest Vessel Count per Asset</t>
+  </si>
+  <si>
+    <t>Activity Used</t>
+  </si>
+  <si>
+    <t>Pivot: Highest Vessels by Asset</t>
+  </si>
+  <si>
+    <t>Max Vessels for Activity</t>
+  </si>
+  <si>
+    <t>First find MAX vessel count for each Asset + Activity</t>
+  </si>
+  <si>
+    <t>Asset result</t>
   </si>
 </sst>
 </file>
@@ -285,7 +341,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -298,11 +354,13 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -317,8 +375,55 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -397,6 +502,42 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5B9BD5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8696B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF63BE7B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF3F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -425,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -455,11 +596,467 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="8" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="74">
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF8696B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF5B9BD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF5B9BD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -470,6 +1067,769 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Coyle, Christopher F SOPUS-PTC/D/MGN" refreshedDate="46204.574663425927" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="17" xr:uid="{AD6C271B-3BB3-4E06-A604-063B19BB3F8E}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A3:C20" sheet="Asset Pivot"/>
+  </cacheSource>
+  <cacheFields count="3">
+    <cacheField name="Asset" numFmtId="0">
+      <sharedItems count="17">
+        <s v="Appomatox, Vito, Olympus"/>
+        <s v="Enchilada"/>
+        <s v="ESA, Ursa"/>
+        <s v="Mars"/>
+        <s v="Noble Voyager"/>
+        <s v="Olympus"/>
+        <s v="Perdido"/>
+        <s v="Perdido/Whale"/>
+        <s v="Pontus"/>
+        <s v="Poseidon"/>
+        <s v="Proteus"/>
+        <s v="Q5000"/>
+        <s v="Salsa"/>
+        <s v="Stena Evolution"/>
+        <s v="Thalassa"/>
+        <s v="Vito"/>
+        <s v="Whale"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Activity Used" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Highest Vessel Count" numFmtId="3">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="2"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="17">
+  <r>
+    <x v="0"/>
+    <s v="EV Run"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Storm Choke well services"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <s v="EV Run"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <s v="A22 Completion"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <s v="Ursa North P013 Top Hole"/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <s v="MB24 Completion"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <s v="GA-23 Deepening"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <s v="EV Run"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <s v="Sisco 001 Drill New Well"/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <s v="LWX 8 Completion"/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="10"/>
+    <s v="VX004 Top Hole"/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="11"/>
+    <s v="Whale 213, Whale 303 PLT Interventions"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="12"/>
+    <s v="Abandonment"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="13"/>
+    <s v="Kaikias KI-2 Drill New Well"/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="14"/>
+    <s v="WS304 Completion"/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="15"/>
+    <s v="WF SURF"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="16"/>
+    <s v="Whale TAR Warehouse Boat"/>
+    <n v="1"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{852E3C97-BA5D-4CB4-A7FF-3E3F88CFC2F1}" name="Pivot_Max_Vessel_Count_By_Asset" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="E3:F20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="18">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" numFmtId="3" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="17">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Highest Vessel Count" fld="2" subtotal="max" baseField="0" baseItem="0" numFmtId="3"/>
+  </dataFields>
+  <formats count="64">
+    <format dxfId="73">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="72">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="71">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="70">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="69">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="68">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="67">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="66">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="65">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="64">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="63">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="62">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="61">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="60">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="59">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="58">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="57">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="56">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="55">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="54">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="53">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="52">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="51">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="50">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="49">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="48">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="47">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="46">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="45">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="44">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="43">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="42">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="41">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="40">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="39">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="38">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="37">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="36">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="35">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="33">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="31">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="30">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="29">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="28">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="27">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="26">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="24">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="23">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="14"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="22">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="14"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="21">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="14"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="20">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="19">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="18">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="17">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="15">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="12">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="11">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2FF6C120-EBF4-413D-8D32-24089D065709}" name="AssetHighestActivityCount" displayName="AssetHighestActivityCount" ref="A3:C20" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A3:C20" xr:uid="{2FF6C120-EBF4-413D-8D32-24089D065709}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{1F54A61A-10F7-4C45-9EA2-6ADEFE1F1301}" name="Asset" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{1E54EFC9-1650-49E1-85C9-337492CBC769}" name="Activity Used" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{9AA64844-40B6-486A-9FD6-5CE8F6ECE903}" name="Highest Vessel Count" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FF1C2CF-4AF0-4C32-81BC-B03A67A5580C}" name="AssetActivityMaxAudit" displayName="AssetActivityMaxAudit" ref="H1:J37" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="H1:J37" xr:uid="{2FF1C2CF-4AF0-4C32-81BC-B03A67A5580C}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{41B3A9FB-86C5-4090-8721-4B881B6E901B}" name="Asset" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{B7F27A0B-B07D-4AF2-B7AF-E9612E04F120}" name="Activity" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{1FD30931-36D0-49C0-89E5-4A1DD1374BE5}" name="Max Vessels for Activity" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -757,21 +2117,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L71"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -800,7 +2160,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
@@ -827,7 +2187,7 @@
       </c>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
@@ -854,7 +2214,7 @@
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>33</v>
       </c>
@@ -881,7 +2241,7 @@
       </c>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -908,7 +2268,7 @@
       </c>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -935,7 +2295,7 @@
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -962,7 +2322,7 @@
       </c>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
@@ -989,7 +2349,7 @@
       </c>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -1016,7 +2376,7 @@
       </c>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
@@ -1043,7 +2403,7 @@
       </c>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
@@ -1070,7 +2430,7 @@
       </c>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
@@ -1097,7 +2457,7 @@
       </c>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
@@ -1108,7 +2468,7 @@
         <v>18</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>26</v>
@@ -1124,7 +2484,7 @@
       </c>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
@@ -1151,7 +2511,7 @@
       </c>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
@@ -1178,7 +2538,7 @@
       </c>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
@@ -1205,7 +2565,7 @@
       </c>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -1232,7 +2592,7 @@
       </c>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>45</v>
       </c>
@@ -1259,7 +2619,7 @@
       </c>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -1286,7 +2646,7 @@
       </c>
       <c r="I19" s="2"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1313,7 +2673,7 @@
       </c>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>13</v>
       </c>
@@ -1340,7 +2700,7 @@
       </c>
       <c r="I21" s="2"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>15</v>
       </c>
@@ -1367,7 +2727,7 @@
       </c>
       <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>17</v>
       </c>
@@ -1378,7 +2738,7 @@
         <v>18</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>35</v>
@@ -1394,7 +2754,7 @@
       </c>
       <c r="I23" s="2"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
@@ -1405,7 +2765,7 @@
         <v>55</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>26</v>
@@ -1421,7 +2781,7 @@
       </c>
       <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>18</v>
       </c>
@@ -1448,7 +2808,7 @@
       </c>
       <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>9</v>
       </c>
@@ -1475,7 +2835,7 @@
       </c>
       <c r="I26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>13</v>
       </c>
@@ -1502,10 +2862,10 @@
       </c>
       <c r="I27" s="2"/>
       <c r="L27" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>15</v>
       </c>
@@ -1532,7 +2892,7 @@
       </c>
       <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>54</v>
       </c>
@@ -1555,11 +2915,11 @@
         <v>46193</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>41</v>
       </c>
@@ -1570,7 +2930,7 @@
         <v>37</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>26</v>
@@ -1586,7 +2946,7 @@
       </c>
       <c r="I30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>9</v>
       </c>
@@ -1609,11 +2969,11 @@
         <v>46203</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>13</v>
       </c>
@@ -1636,11 +2996,11 @@
         <v>46203</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I32" s="2"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>15</v>
       </c>
@@ -1663,11 +3023,11 @@
         <v>46203</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I33" s="2"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>43</v>
       </c>
@@ -1678,7 +3038,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>26</v>
@@ -1694,88 +3054,88 @@
       </c>
       <c r="I34" s="2"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="2">
+        <v>2</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F35" s="4">
+        <v>46152</v>
+      </c>
+      <c r="G35" s="4">
+        <v>46215</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I35" s="2"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B35" s="2">
-        <v>1</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="B36" s="2">
+        <v>1</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D35" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="E35" s="9" t="s">
+      <c r="D36" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E36" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F35" s="4">
+      <c r="F36" s="4">
         <v>46204</v>
       </c>
-      <c r="G35" s="4">
+      <c r="G36" s="4">
         <v>46222</v>
       </c>
-      <c r="H35" s="24" t="s">
+      <c r="H36" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
+      <c r="I36" s="2"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B36" s="2">
-        <v>2</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F36" s="4">
-        <v>46193</v>
-      </c>
-      <c r="G36" s="4">
-        <v>46227</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I36" s="2"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="B37" s="2">
         <v>2</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>26</v>
       </c>
       <c r="F37" s="4">
-        <v>46152</v>
+        <v>46194</v>
       </c>
       <c r="G37" s="4">
-        <v>46213</v>
+        <v>46234</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I37" s="2"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>22</v>
       </c>
@@ -1795,49 +3155,49 @@
         <v>46191</v>
       </c>
       <c r="G38" s="4">
-        <v>46232</v>
+        <v>46238</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I38" s="2"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B39" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>26</v>
+        <v>11</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F39" s="4">
-        <v>46190</v>
+        <v>46204</v>
       </c>
       <c r="G39" s="4">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="I39" s="2"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B40" s="2">
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>11</v>
@@ -1856,15 +3216,15 @@
       </c>
       <c r="I40" s="2"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B41" s="2">
         <v>1</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>11</v>
@@ -1883,169 +3243,169 @@
       </c>
       <c r="I41" s="2"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B42" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>11</v>
+        <v>67</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="F42" s="4">
-        <v>46204</v>
+        <v>46191</v>
       </c>
       <c r="G42" s="4">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I42" s="2"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="B43" s="2">
         <v>2</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>30</v>
+        <v>80</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>35</v>
       </c>
       <c r="F43" s="4">
-        <v>46225</v>
+        <v>46215</v>
       </c>
       <c r="G43" s="4">
-        <v>46240</v>
+        <v>46245</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I43" s="2"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="B44" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="D44" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="F44" s="4">
-        <v>46213</v>
+        <v>46194</v>
       </c>
       <c r="G44" s="4">
-        <v>46243</v>
-      </c>
-      <c r="H44" s="2" t="s">
+        <v>46252</v>
+      </c>
+      <c r="H44" s="24" t="s">
         <v>12</v>
       </c>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="B45" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="E45" s="8" t="s">
         <v>30</v>
       </c>
       <c r="F45" s="4">
-        <v>46242</v>
+        <v>46225</v>
       </c>
       <c r="G45" s="4">
-        <v>46249</v>
+        <v>46252</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="B46" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D46" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="E46" s="7" t="s">
-        <v>26</v>
+        <v>18</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="F46" s="4">
-        <v>46194</v>
+        <v>46245</v>
       </c>
       <c r="G46" s="4">
         <v>46252</v>
       </c>
-      <c r="H46" s="24" t="s">
+      <c r="H46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="B47" s="2">
         <v>2</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>26</v>
       </c>
       <c r="F47" s="4">
-        <v>46240</v>
+        <v>46234</v>
       </c>
       <c r="G47" s="4">
-        <v>46265</v>
+        <v>46268</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I47" s="2"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>9</v>
       </c>
@@ -2072,7 +3432,7 @@
       </c>
       <c r="I48" s="2"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>13</v>
       </c>
@@ -2099,7 +3459,7 @@
       </c>
       <c r="I49" s="2"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>15</v>
       </c>
@@ -2126,69 +3486,69 @@
       </c>
       <c r="I50" s="2"/>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="B51" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" s="3" t="s">
-        <v>11</v>
+        <v>72</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="F51" s="4">
-        <v>46266</v>
+        <v>46252</v>
       </c>
       <c r="G51" s="4">
-        <v>46295</v>
+        <v>46278</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I51" s="2"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B52" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>11</v>
+        <v>83</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="F52" s="4">
-        <v>46266</v>
+        <v>46252</v>
       </c>
       <c r="G52" s="4">
-        <v>46295</v>
+        <v>46279</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I52" s="2"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B53" s="2">
         <v>1</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>11</v>
@@ -2207,15 +3567,15 @@
       </c>
       <c r="I53" s="2"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B54" s="2">
         <v>1</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>11</v>
@@ -2224,25 +3584,25 @@
         <v>11</v>
       </c>
       <c r="F54" s="4">
-        <v>46296</v>
+        <v>46266</v>
       </c>
       <c r="G54" s="4">
-        <v>46326</v>
+        <v>46295</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I54" s="2"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B55" s="2">
         <v>1</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>11</v>
@@ -2251,79 +3611,79 @@
         <v>11</v>
       </c>
       <c r="F55" s="4">
-        <v>46296</v>
+        <v>46266</v>
       </c>
       <c r="G55" s="4">
-        <v>46326</v>
+        <v>46295</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I55" s="2"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="B56" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>11</v>
+        <v>84</v>
+      </c>
+      <c r="E56" s="25" t="s">
+        <v>35</v>
       </c>
       <c r="F56" s="4">
-        <v>46296</v>
+        <v>46278</v>
       </c>
       <c r="G56" s="4">
-        <v>46326</v>
+        <v>46298</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I56" s="2"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="B57" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>11</v>
+        <v>85</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="F57" s="4">
-        <v>46327</v>
+        <v>46298</v>
       </c>
       <c r="G57" s="4">
-        <v>46356</v>
+        <v>46318</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I57" s="2"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B58" s="2">
         <v>1</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>11</v>
@@ -2332,25 +3692,25 @@
         <v>11</v>
       </c>
       <c r="F58" s="4">
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="G58" s="4">
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I58" s="2"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B59" s="2">
         <v>1</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>11</v>
@@ -2359,25 +3719,25 @@
         <v>11</v>
       </c>
       <c r="F59" s="4">
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="G59" s="4">
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I59" s="2"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B60" s="2">
         <v>1</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>11</v>
@@ -2386,25 +3746,25 @@
         <v>11</v>
       </c>
       <c r="F60" s="4">
-        <v>46023</v>
+        <v>46296</v>
       </c>
       <c r="G60" s="4">
-        <v>46386</v>
+        <v>46326</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I60" s="2"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B61" s="2">
         <v>1</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>11</v>
@@ -2413,25 +3773,25 @@
         <v>11</v>
       </c>
       <c r="F61" s="4">
-        <v>46023</v>
+        <v>46327</v>
       </c>
       <c r="G61" s="4">
-        <v>46386</v>
+        <v>46356</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I61" s="2"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B62" s="2">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>11</v>
@@ -2440,25 +3800,25 @@
         <v>11</v>
       </c>
       <c r="F62" s="4">
-        <v>46023</v>
+        <v>46327</v>
       </c>
       <c r="G62" s="4">
-        <v>46386</v>
+        <v>46356</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I62" s="2"/>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B63" s="2">
         <v>1</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>11</v>
@@ -2467,17 +3827,17 @@
         <v>11</v>
       </c>
       <c r="F63" s="4">
-        <v>46357</v>
+        <v>46327</v>
       </c>
       <c r="G63" s="4">
-        <v>46387</v>
+        <v>46356</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I63" s="2"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>13</v>
       </c>
@@ -2494,25 +3854,25 @@
         <v>11</v>
       </c>
       <c r="F64" s="4">
-        <v>46357</v>
+        <v>46023</v>
       </c>
       <c r="G64" s="4">
-        <v>46387</v>
+        <v>46386</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I64" s="2"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B65" s="2">
         <v>1</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>11</v>
@@ -2521,46 +3881,46 @@
         <v>11</v>
       </c>
       <c r="F65" s="4">
-        <v>46357</v>
+        <v>46023</v>
       </c>
       <c r="G65" s="4">
-        <v>46387</v>
+        <v>46386</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I65" s="2"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="B66" s="2">
         <v>1</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>39</v>
+        <v>11</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F66" s="4">
-        <v>46266</v>
+        <v>46023</v>
       </c>
       <c r="G66" s="4">
-        <v>46387</v>
+        <v>46386</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I66" s="2"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="B67" s="2">
         <v>1</v>
@@ -2569,13 +3929,13 @@
         <v>10</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F67" s="4">
-        <v>46266</v>
+        <v>46357</v>
       </c>
       <c r="G67" s="4">
         <v>46387</v>
@@ -2585,10 +3945,118 @@
       </c>
       <c r="I67" s="2"/>
     </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B68" s="2">
+        <v>1</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68" s="4">
+        <v>46357</v>
+      </c>
+      <c r="G68" s="4">
+        <v>46387</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I68" s="2"/>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B69" s="2">
+        <v>1</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F69" s="4">
+        <v>46357</v>
+      </c>
+      <c r="G69" s="4">
+        <v>46387</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I69" s="2"/>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B70" s="2">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E70" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F70" s="4">
+        <v>46266</v>
+      </c>
+      <c r="G70" s="4">
+        <v>46387</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I70" s="2"/>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B71" s="2">
+        <v>1</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F71" s="4">
+        <v>46266</v>
+      </c>
+      <c r="G71" s="4">
+        <v>46387</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I71" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I67" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I68">
-      <sortCondition ref="G1"/>
+  <autoFilter ref="A1:I71" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A30:I71">
+      <sortCondition ref="G1:G71"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2598,13 +4066,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>58</v>
       </c>
@@ -2612,7 +4080,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>11</v>
       </c>
@@ -2620,7 +4088,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>30</v>
       </c>
@@ -2628,7 +4096,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>26</v>
       </c>
@@ -2636,7 +4104,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>35</v>
       </c>
@@ -2644,7 +4112,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
         <v>63</v>
       </c>
@@ -2652,33 +4120,919 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>39</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CE295E-4F55-4292-8842-FF5EFD53550D}">
+  <dimension ref="A1:J37"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="38.6640625" style="28" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.33203125" style="28" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" s="35"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="26"/>
+      <c r="E3" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="32">
+        <v>1</v>
+      </c>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="32">
+        <v>1</v>
+      </c>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="32">
+        <v>1</v>
+      </c>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="32">
+        <v>1</v>
+      </c>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="32">
+        <v>1</v>
+      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="32">
+        <v>1</v>
+      </c>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="32">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="32">
+        <v>1</v>
+      </c>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="J7" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="31">
+        <v>2</v>
+      </c>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="31">
+        <v>2</v>
+      </c>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="I8" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="J8" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="32">
+        <v>1</v>
+      </c>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="32">
+        <v>1</v>
+      </c>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="I9" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="J9" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="32">
+        <v>1</v>
+      </c>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="32">
+        <v>1</v>
+      </c>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="J10" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="32">
+        <v>1</v>
+      </c>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="32">
+        <v>1</v>
+      </c>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="31">
+        <v>2</v>
+      </c>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="31">
+        <v>2</v>
+      </c>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="J12" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="31">
+        <v>2</v>
+      </c>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="31">
+        <v>2</v>
+      </c>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="I13" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="31">
+        <v>2</v>
+      </c>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="31">
+        <v>2</v>
+      </c>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="I14" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="J14" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="32">
+        <v>1</v>
+      </c>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="32">
+        <v>1</v>
+      </c>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="J15" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="32">
+        <v>1</v>
+      </c>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" s="32">
+        <v>1</v>
+      </c>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="J16" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="31">
+        <v>2</v>
+      </c>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="31">
+        <v>2</v>
+      </c>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="J17" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="31">
+        <v>2</v>
+      </c>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="31">
+        <v>2</v>
+      </c>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="32">
+        <v>1</v>
+      </c>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="32">
+        <v>1</v>
+      </c>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="J19" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="32">
+        <v>1</v>
+      </c>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="32">
+        <v>1</v>
+      </c>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="J20" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="26"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="J21" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="26"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="J22" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="36"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="J23" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="J24" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="26"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="J25" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="26"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="J26" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="26"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="I27" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="J27" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="I28" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="J28" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="26"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="I29" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="J29" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="26"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="J30" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="26"/>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I31" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="J31" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="26"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I32" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="J32" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="26"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I33" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="J33" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="26"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I34" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="J34" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="26"/>
+      <c r="B35" s="26"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="I35" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="J35" s="29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="I36" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="J36" s="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="26"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="I37" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="J37" s="29">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B23:C24"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update Spot Hire workbook - July 9, 2026
</commit_message>
<xml_diff>
--- a/Spot_Hire_Update_20260611.xlsx
+++ b/Spot_Hire_Update_20260611.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://my.shell.com/personal/chris_coyle_shell_com/Documents/VS Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="618" documentId="11_C9588FE751541D8D1C6E4DD53657CAD1CCF10B9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CEB083B-588E-4873-9E7E-A46681CBC432}"/>
+  <xr:revisionPtr revIDLastSave="699" documentId="11_C9588FE751541D8D1C6E4DD53657CAD1CCF10B9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE93B0A7-23B7-4B59-828B-B46CFE484AD5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spot Hire Update" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Asset Pivot" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Spot Hire Update'!$A$1:$I$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Spot Hire Update'!$A$1:$I$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="100">
   <si>
     <t>Asset</t>
   </si>
@@ -332,6 +332,15 @@
   </si>
   <si>
     <t>Asset result</t>
+  </si>
+  <si>
+    <t>NVOY Arrival and Commisioning at Deep Sleep Dummy Well</t>
+  </si>
+  <si>
+    <t>Deep Sleep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top Hole </t>
   </si>
 </sst>
 </file>
@@ -539,7 +548,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -562,11 +571,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -574,7 +596,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -614,6 +635,9 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2117,21 +2141,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L71"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L73"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2160,7 +2184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
@@ -2173,7 +2197,7 @@
       <c r="D2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F2" s="4">
@@ -2187,7 +2211,7 @@
       </c>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
@@ -2200,7 +2224,7 @@
       <c r="D3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F3" s="4">
@@ -2214,7 +2238,7 @@
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>33</v>
       </c>
@@ -2227,7 +2251,7 @@
       <c r="D4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F4" s="4">
@@ -2241,7 +2265,7 @@
       </c>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -2254,7 +2278,7 @@
       <c r="D5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>30</v>
       </c>
       <c r="F5" s="4">
@@ -2268,7 +2292,7 @@
       </c>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -2281,7 +2305,7 @@
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F6" s="4">
@@ -2295,7 +2319,7 @@
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -2322,7 +2346,7 @@
       </c>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
@@ -2335,7 +2359,7 @@
       <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F8" s="4">
@@ -2349,7 +2373,7 @@
       </c>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -2376,7 +2400,7 @@
       </c>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
@@ -2403,7 +2427,7 @@
       </c>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
@@ -2430,12 +2454,12 @@
       </c>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B12" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>23</v>
@@ -2443,7 +2467,7 @@
       <c r="D12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F12" s="4">
@@ -2457,7 +2481,7 @@
       </c>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
@@ -2470,7 +2494,7 @@
       <c r="D13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F13" s="4">
@@ -2484,7 +2508,7 @@
       </c>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
@@ -2497,7 +2521,7 @@
       <c r="D14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="9" t="s">
         <v>39</v>
       </c>
       <c r="F14" s="4">
@@ -2511,7 +2535,7 @@
       </c>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
@@ -2538,7 +2562,7 @@
       </c>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
@@ -2565,7 +2589,7 @@
       </c>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -2592,7 +2616,7 @@
       </c>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>45</v>
       </c>
@@ -2605,7 +2629,7 @@
       <c r="D18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>69</v>
       </c>
       <c r="F18" s="4">
@@ -2619,34 +2643,34 @@
       </c>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="2">
-        <v>1</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="B19" s="36">
+        <v>1</v>
+      </c>
+      <c r="C19" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="38">
         <v>46218</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="38">
         <v>46142</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="I19" s="36"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -2673,7 +2697,7 @@
       </c>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>13</v>
       </c>
@@ -2700,7 +2724,7 @@
       </c>
       <c r="I21" s="2"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>15</v>
       </c>
@@ -2727,7 +2751,7 @@
       </c>
       <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>17</v>
       </c>
@@ -2740,7 +2764,7 @@
       <c r="D23" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F23" s="4">
@@ -2754,7 +2778,7 @@
       </c>
       <c r="I23" s="2"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
@@ -2767,7 +2791,7 @@
       <c r="D24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F24" s="4">
@@ -2781,7 +2805,7 @@
       </c>
       <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>18</v>
       </c>
@@ -2794,7 +2818,7 @@
       <c r="D25" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F25" s="4">
@@ -2808,7 +2832,7 @@
       </c>
       <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>9</v>
       </c>
@@ -2835,7 +2859,7 @@
       </c>
       <c r="I26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>13</v>
       </c>
@@ -2865,7 +2889,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>15</v>
       </c>
@@ -2892,7 +2916,7 @@
       </c>
       <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>54</v>
       </c>
@@ -2905,7 +2929,7 @@
       <c r="D29" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F29" s="4">
@@ -2919,7 +2943,7 @@
       </c>
       <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>41</v>
       </c>
@@ -2929,10 +2953,10 @@
       <c r="C30" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D30" s="23" t="s">
+      <c r="D30" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F30" s="4">
@@ -2946,7 +2970,7 @@
       </c>
       <c r="I30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>9</v>
       </c>
@@ -2973,7 +2997,7 @@
       </c>
       <c r="I31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>13</v>
       </c>
@@ -3000,7 +3024,7 @@
       </c>
       <c r="I32" s="2"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>15</v>
       </c>
@@ -3027,7 +3051,7 @@
       </c>
       <c r="I33" s="2"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>43</v>
       </c>
@@ -3037,10 +3061,10 @@
       <c r="C34" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D34" s="23" t="s">
+      <c r="D34" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F34" s="4">
@@ -3054,7 +3078,7 @@
       </c>
       <c r="I34" s="2"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>17</v>
       </c>
@@ -3067,21 +3091,21 @@
       <c r="D35" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F35" s="4">
         <v>46152</v>
       </c>
       <c r="G35" s="4">
-        <v>46215</v>
+        <v>46218</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I35" s="2"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>43</v>
       </c>
@@ -3091,10 +3115,10 @@
       <c r="C36" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D36" s="23" t="s">
+      <c r="D36" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F36" s="4">
@@ -3103,12 +3127,12 @@
       <c r="G36" s="4">
         <v>46222</v>
       </c>
-      <c r="H36" s="24" t="s">
+      <c r="H36" s="23" t="s">
         <v>12</v>
       </c>
       <c r="I36" s="2"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>54</v>
       </c>
@@ -3121,21 +3145,21 @@
       <c r="D37" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E37" s="7" t="s">
+      <c r="E37" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F37" s="4">
         <v>46194</v>
       </c>
       <c r="G37" s="4">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I37" s="2"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>22</v>
       </c>
@@ -3148,21 +3172,21 @@
       <c r="D38" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F38" s="4">
         <v>46191</v>
       </c>
       <c r="G38" s="4">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I38" s="2"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>9</v>
       </c>
@@ -3189,7 +3213,7 @@
       </c>
       <c r="I39" s="2"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>13</v>
       </c>
@@ -3216,7 +3240,7 @@
       </c>
       <c r="I40" s="2"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>15</v>
       </c>
@@ -3243,7 +3267,7 @@
       </c>
       <c r="I41" s="2"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>22</v>
       </c>
@@ -3256,7 +3280,7 @@
       <c r="D42" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F42" s="4">
@@ -3270,7 +3294,7 @@
       </c>
       <c r="I42" s="2"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>17</v>
       </c>
@@ -3283,21 +3307,21 @@
       <c r="D43" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F43" s="4">
-        <v>46215</v>
+        <v>46218</v>
       </c>
       <c r="G43" s="4">
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I43" s="2"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>41</v>
       </c>
@@ -3307,10 +3331,10 @@
       <c r="C44" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D44" s="23" t="s">
+      <c r="D44" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F44" s="4">
@@ -3319,128 +3343,128 @@
       <c r="G44" s="4">
         <v>46252</v>
       </c>
-      <c r="H44" s="24" t="s">
+      <c r="H44" s="23" t="s">
         <v>12</v>
       </c>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B45" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>30</v>
+        <v>98</v>
+      </c>
+      <c r="D45" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>99</v>
       </c>
       <c r="F45" s="4">
         <v>46225</v>
       </c>
       <c r="G45" s="4">
-        <v>46252</v>
-      </c>
-      <c r="H45" s="2" t="s">
+        <v>46247</v>
+      </c>
+      <c r="H45" s="23" t="s">
         <v>12</v>
       </c>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="B46" s="2">
         <v>3</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E46" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E46" s="7" t="s">
         <v>30</v>
       </c>
       <c r="F46" s="4">
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="G46" s="4">
-        <v>46252</v>
+        <v>46258</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="B47" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F47" s="4">
-        <v>46234</v>
+        <v>46248</v>
       </c>
       <c r="G47" s="4">
-        <v>46268</v>
+        <v>46255</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I47" s="2"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="B48" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>11</v>
+        <v>87</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="F48" s="4">
         <v>46235</v>
       </c>
       <c r="G48" s="4">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I48" s="2"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B49" s="2">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>11</v>
@@ -3459,15 +3483,15 @@
       </c>
       <c r="I49" s="2"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B50" s="2">
         <v>1</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>11</v>
@@ -3486,96 +3510,96 @@
       </c>
       <c r="I50" s="2"/>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="B51" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>26</v>
+        <v>11</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F51" s="4">
-        <v>46252</v>
+        <v>46235</v>
       </c>
       <c r="G51" s="4">
-        <v>46278</v>
+        <v>46265</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I51" s="2"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="B52" s="2">
         <v>2</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E52" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F52" s="4">
-        <v>46252</v>
+        <v>46258</v>
       </c>
       <c r="G52" s="4">
-        <v>46279</v>
+        <v>46284</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I52" s="2"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B53" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>11</v>
+        <v>83</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="F53" s="4">
-        <v>46266</v>
+        <v>46255</v>
       </c>
       <c r="G53" s="4">
-        <v>46295</v>
+        <v>46282</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I53" s="2"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B54" s="2">
         <v>1</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>11</v>
@@ -3594,15 +3618,15 @@
       </c>
       <c r="I54" s="2"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B55" s="2">
         <v>1</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>11</v>
@@ -3621,34 +3645,34 @@
       </c>
       <c r="I55" s="2"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="B56" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E56" s="25" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F56" s="4">
-        <v>46278</v>
+        <v>46266</v>
       </c>
       <c r="G56" s="4">
-        <v>46298</v>
+        <v>46295</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I56" s="2"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>70</v>
       </c>
@@ -3656,61 +3680,61 @@
         <v>2</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E57" s="7" t="s">
-        <v>26</v>
+        <v>84</v>
+      </c>
+      <c r="E57" s="24" t="s">
+        <v>35</v>
       </c>
       <c r="F57" s="4">
-        <v>46298</v>
+        <v>46284</v>
       </c>
       <c r="G57" s="4">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I57" s="2"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="B58" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>11</v>
+        <v>85</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="F58" s="4">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="G58" s="4">
-        <v>46326</v>
+        <v>46324</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I58" s="2"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B59" s="2">
         <v>1</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>11</v>
@@ -3729,15 +3753,15 @@
       </c>
       <c r="I59" s="2"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B60" s="2">
         <v>1</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>11</v>
@@ -3756,15 +3780,15 @@
       </c>
       <c r="I60" s="2"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B61" s="2">
         <v>1</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>11</v>
@@ -3773,25 +3797,25 @@
         <v>11</v>
       </c>
       <c r="F61" s="4">
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="G61" s="4">
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I61" s="2"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B62" s="2">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>11</v>
@@ -3810,15 +3834,15 @@
       </c>
       <c r="I62" s="2"/>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B63" s="2">
         <v>1</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>11</v>
@@ -3837,15 +3861,15 @@
       </c>
       <c r="I63" s="2"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B64" s="2">
         <v>1</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>11</v>
@@ -3854,17 +3878,17 @@
         <v>11</v>
       </c>
       <c r="F64" s="4">
-        <v>46023</v>
+        <v>46327</v>
       </c>
       <c r="G64" s="4">
-        <v>46386</v>
+        <v>46356</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I64" s="2"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>13</v>
       </c>
@@ -3891,15 +3915,15 @@
       </c>
       <c r="I65" s="2"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B66" s="2">
         <v>1</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>11</v>
@@ -3918,15 +3942,15 @@
       </c>
       <c r="I66" s="2"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B67" s="2">
         <v>1</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>11</v>
@@ -3935,25 +3959,25 @@
         <v>11</v>
       </c>
       <c r="F67" s="4">
-        <v>46357</v>
+        <v>46023</v>
       </c>
       <c r="G67" s="4">
-        <v>46387</v>
+        <v>46386</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I67" s="2"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B68" s="2">
         <v>1</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>11</v>
@@ -3972,15 +3996,15 @@
       </c>
       <c r="I68" s="2"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B69" s="2">
         <v>1</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>11</v>
@@ -3999,24 +4023,24 @@
       </c>
       <c r="I69" s="2"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="B70" s="2">
         <v>1</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>39</v>
+        <v>11</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F70" s="4">
-        <v>46266</v>
+        <v>46357</v>
       </c>
       <c r="G70" s="4">
         <v>46387</v>
@@ -4026,9 +4050,9 @@
       </c>
       <c r="I70" s="2"/>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B71" s="2">
         <v>1</v>
@@ -4037,10 +4061,10 @@
         <v>10</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>25</v>
+        <v>50</v>
+      </c>
+      <c r="E71" s="9" t="s">
+        <v>39</v>
       </c>
       <c r="F71" s="4">
         <v>46266</v>
@@ -4053,10 +4077,64 @@
       </c>
       <c r="I71" s="2"/>
     </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B72" s="2">
+        <v>1</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F72" s="4">
+        <v>46266</v>
+      </c>
+      <c r="G72" s="4">
+        <v>46387</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I72" s="2"/>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B73" s="2">
+        <v>2</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F73" s="4">
+        <v>46206</v>
+      </c>
+      <c r="G73" s="4">
+        <v>46219</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I73" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I71" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A30:I71">
-      <sortCondition ref="G1:G71"/>
+  <autoFilter ref="A1:I73" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A30:I72">
+      <sortCondition ref="G1:G72"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4066,82 +4144,82 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
         <v>11</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
         <v>30</v>
       </c>
       <c r="C3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
         <v>26</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
         <v>35</v>
       </c>
       <c r="C5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
         <v>63</v>
       </c>
       <c r="C6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
         <v>39</v>
       </c>
     </row>
@@ -4153,872 +4231,872 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CE295E-4F55-4292-8842-FF5EFD53550D}">
   <dimension ref="A1:J37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" style="28" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="38.6640625" style="28" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.33203125" style="28" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" style="27" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="38.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.28515625" style="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="35" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="35"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26" t="s">
+      <c r="F1" s="34"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="29" t="s">
+      <c r="J1" s="28" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="25"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+      <c r="I2" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27" t="s">
+      <c r="D3" s="25"/>
+      <c r="E3" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="33" t="s">
+      <c r="F3" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26" t="s">
+      <c r="G3" s="25"/>
+      <c r="H3" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="26" t="s">
+      <c r="I3" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="J3" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
+      <c r="J3" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="32">
-        <v>1</v>
-      </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26" t="s">
+      <c r="B4" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="31">
+        <v>1</v>
+      </c>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="32">
-        <v>1</v>
-      </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26" t="s">
+      <c r="F4" s="31">
+        <v>1</v>
+      </c>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="J4" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
+      <c r="I4" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="32">
-        <v>1</v>
-      </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26" t="s">
+      <c r="C5" s="31">
+        <v>1</v>
+      </c>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="32">
-        <v>1</v>
-      </c>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26" t="s">
+      <c r="F5" s="31">
+        <v>1</v>
+      </c>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="26" t="s">
+      <c r="I5" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
+      <c r="J5" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="32">
-        <v>1</v>
-      </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26" t="s">
+      <c r="B6" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="31">
+        <v>1</v>
+      </c>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="32">
-        <v>1</v>
-      </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26" t="s">
+      <c r="F6" s="31">
+        <v>1</v>
+      </c>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="26" t="s">
+      <c r="I6" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="J6" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+      <c r="J6" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="32">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26" t="s">
+      <c r="C7" s="31">
+        <v>1</v>
+      </c>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="F7" s="32">
-        <v>1</v>
-      </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26" t="s">
+      <c r="F7" s="31">
+        <v>1</v>
+      </c>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="26" t="s">
+      <c r="I7" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
+      <c r="J7" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="30">
         <v>2</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26" t="s">
+      <c r="D8" s="25"/>
+      <c r="E8" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="30">
         <v>2</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26" t="s">
+      <c r="G8" s="25"/>
+      <c r="H8" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="26" t="s">
+      <c r="I8" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="J8" s="29">
+      <c r="J8" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="26" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="32">
-        <v>1</v>
-      </c>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26" t="s">
+      <c r="C9" s="31">
+        <v>1</v>
+      </c>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="32">
-        <v>1</v>
-      </c>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26" t="s">
+      <c r="F9" s="31">
+        <v>1</v>
+      </c>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="I9" s="26" t="s">
+      <c r="I9" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="29">
+      <c r="J9" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="26" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="32">
-        <v>1</v>
-      </c>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26" t="s">
+      <c r="C10" s="31">
+        <v>1</v>
+      </c>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="32">
-        <v>1</v>
-      </c>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26" t="s">
+      <c r="F10" s="31">
+        <v>1</v>
+      </c>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="I10" s="26" t="s">
+      <c r="I10" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="J10" s="29">
+      <c r="J10" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="26" t="s">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="32">
-        <v>1</v>
-      </c>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26" t="s">
+      <c r="B11" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="31">
+        <v>1</v>
+      </c>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="32">
-        <v>1</v>
-      </c>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26" t="s">
+      <c r="F11" s="31">
+        <v>1</v>
+      </c>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="I11" s="26" t="s">
+      <c r="I11" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="J11" s="29">
+      <c r="J11" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="30">
         <v>2</v>
       </c>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26" t="s">
+      <c r="D12" s="25"/>
+      <c r="E12" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="30">
         <v>2</v>
       </c>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26" t="s">
+      <c r="G12" s="25"/>
+      <c r="H12" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="I12" s="26" t="s">
+      <c r="I12" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="J12" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="26" t="s">
+      <c r="J12" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="30">
         <v>2</v>
       </c>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26" t="s">
+      <c r="D13" s="25"/>
+      <c r="E13" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="30">
         <v>2</v>
       </c>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26" t="s">
+      <c r="G13" s="25"/>
+      <c r="H13" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="I13" s="26" t="s">
+      <c r="I13" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="J13" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+      <c r="J13" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="30">
         <v>2</v>
       </c>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26" t="s">
+      <c r="D14" s="25"/>
+      <c r="E14" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="30">
         <v>2</v>
       </c>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26" t="s">
+      <c r="G14" s="25"/>
+      <c r="H14" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="I14" s="26" t="s">
+      <c r="I14" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+      <c r="J14" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="32">
-        <v>1</v>
-      </c>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26" t="s">
+      <c r="C15" s="31">
+        <v>1</v>
+      </c>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="32">
-        <v>1</v>
-      </c>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26" t="s">
+      <c r="F15" s="31">
+        <v>1</v>
+      </c>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="26" t="s">
+      <c r="I15" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="J15" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+      <c r="J15" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="32">
-        <v>1</v>
-      </c>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26" t="s">
+      <c r="C16" s="31">
+        <v>1</v>
+      </c>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="32">
-        <v>1</v>
-      </c>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26" t="s">
+      <c r="F16" s="31">
+        <v>1</v>
+      </c>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="J16" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
+      <c r="I16" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="J16" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="30">
         <v>2</v>
       </c>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26" t="s">
+      <c r="D17" s="25"/>
+      <c r="E17" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="F17" s="31">
+      <c r="F17" s="30">
         <v>2</v>
       </c>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26" t="s">
+      <c r="G17" s="25"/>
+      <c r="H17" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="I17" s="26" t="s">
+      <c r="I17" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="J17" s="29">
+      <c r="J17" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="26" t="s">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="30">
         <v>2</v>
       </c>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26" t="s">
+      <c r="D18" s="25"/>
+      <c r="E18" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="31">
+      <c r="F18" s="30">
         <v>2</v>
       </c>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26" t="s">
+      <c r="G18" s="25"/>
+      <c r="H18" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="26" t="s">
+      <c r="I18" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="J18" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
+      <c r="J18" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="32">
-        <v>1</v>
-      </c>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26" t="s">
+      <c r="C19" s="31">
+        <v>1</v>
+      </c>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="32">
-        <v>1</v>
-      </c>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26" t="s">
+      <c r="F19" s="31">
+        <v>1</v>
+      </c>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="I19" s="26" t="s">
+      <c r="I19" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="J19" s="29">
+      <c r="J19" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="32">
-        <v>1</v>
-      </c>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26" t="s">
+      <c r="C20" s="31">
+        <v>1</v>
+      </c>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="32">
-        <v>1</v>
-      </c>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26" t="s">
+      <c r="F20" s="31">
+        <v>1</v>
+      </c>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="26" t="s">
+      <c r="I20" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="26"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26" t="s">
+      <c r="J20" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="25"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="26" t="s">
+      <c r="I21" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="J21" s="29">
+      <c r="J21" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="26"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26" t="s">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="26" t="s">
+      <c r="I22" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="J22" s="29">
+      <c r="J22" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="30" t="s">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="36"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26" t="s">
+      <c r="C23" s="35"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I23" s="26" t="s">
+      <c r="I23" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="J23" s="29">
+      <c r="J23" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="29"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26" t="s">
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="26" t="s">
+      <c r="I24" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="J24" s="29">
+      <c r="J24" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="26"/>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="25"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I25" s="26" t="s">
+      <c r="I25" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="J25" s="29">
+      <c r="J25" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="26"/>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="25"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I26" s="26" t="s">
+      <c r="I26" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="J26" s="29">
+      <c r="J26" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="26"/>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="25"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="I27" s="26" t="s">
+      <c r="I27" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="J27" s="29">
+      <c r="J27" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="26"/>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="I28" s="26" t="s">
+      <c r="I28" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="J28" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26" t="s">
+      <c r="J28" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="I29" s="26" t="s">
+      <c r="I29" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="J29" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="26"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26" t="s">
+      <c r="J29" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="25"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="I30" s="26" t="s">
+      <c r="I30" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="J30" s="29">
+      <c r="J30" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26" t="s">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="I31" s="26" t="s">
+      <c r="I31" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="J31" s="29">
+      <c r="J31" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26" t="s">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="25"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="I32" s="26" t="s">
+      <c r="I32" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="J32" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26" t="s">
+      <c r="J32" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="I33" s="26" t="s">
+      <c r="I33" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="J33" s="29">
+      <c r="J33" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" s="26"/>
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="29"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26" t="s">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="25"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="I34" s="26" t="s">
+      <c r="I34" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="J34" s="29">
+      <c r="J34" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="26"/>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="29"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26" t="s">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="25"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I35" s="26" t="s">
+      <c r="I35" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="J35" s="29">
+      <c r="J35" s="28">
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="26"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="29"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26" t="s">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="25"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="I36" s="26" t="s">
+      <c r="I36" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="J36" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="26"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26" t="s">
+      <c r="J36" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="25"/>
+      <c r="B37" s="25"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="I37" s="26" t="s">
+      <c r="I37" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="J37" s="29">
+      <c r="J37" s="28">
         <v>1</v>
       </c>
     </row>

</xml_diff>